<commit_message>
corpus(ssrm): Griffiths & Lane Ex.6 — final figures + at-failure solution sidecars
Both cases reproduce their locks exactly (dry 2.403->2.40, full 1.858) with
the at-failure mechanism captured; failure sidecars persisted for solve-free
re-renders. Ex.6 builder already carried the paper's SI E'=1e5 kPa, nu'=0.3
(no stiffness change needed). Completes the Griffiths & Lane page re-render
(Examples 1-6) begun after the deformation-figure overhaul.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/fem/files/xslope_griffiths6_dry.xlsx
+++ b/docs/fem/files/xslope_griffiths6_dry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53F4FFA-A72E-9849-8C3B-3C3A51EB7D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920EFD39-E0D9-5841-8A8C-9199354BBCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="2900" windowWidth="42700" windowHeight="22800" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="35040" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="240">
   <si>
     <t>X</t>
   </si>
@@ -305,9 +305,6 @@
     <t>s(f)</t>
   </si>
   <si>
-    <t>Base Values</t>
-  </si>
-  <si>
     <t>Standard Deviations</t>
   </si>
   <si>
@@ -450,9 +447,6 @@
     <t>max depth defines the elevation of a horizontal line that is treated as the bottom of the profile</t>
   </si>
   <si>
-    <t>Head:</t>
-  </si>
-  <si>
     <t>seep bc</t>
   </si>
   <si>
@@ -465,9 +459,6 @@
     <t>XSLOPE Input Template</t>
   </si>
   <si>
-    <t>Stress</t>
-  </si>
-  <si>
     <t>E</t>
   </si>
   <si>
@@ -558,40 +549,10 @@
     <t>Distributed Load #6</t>
   </si>
   <si>
-    <t>Specified Head #1</t>
-  </si>
-  <si>
-    <t>Specified Head #2</t>
-  </si>
-  <si>
-    <t>Specified Head #3</t>
-  </si>
-  <si>
-    <t>Specified Head #4</t>
-  </si>
-  <si>
-    <t>Specified Head #5</t>
-  </si>
-  <si>
     <t>Exit Face</t>
   </si>
   <si>
-    <t>Specified Head #1 (2)</t>
-  </si>
-  <si>
     <t>Exit Face (2)</t>
-  </si>
-  <si>
-    <t>Specified Head #2 (2)</t>
-  </si>
-  <si>
-    <t>Specified Head #3 (2)</t>
-  </si>
-  <si>
-    <t>Specified Head #4 (2)</t>
-  </si>
-  <si>
-    <t>Specified Head #5 (2)</t>
   </si>
   <si>
     <t>Distributed Load #1 (2)</t>
@@ -758,16 +719,7 @@
     <t>linear front model (kr0,h0)</t>
   </si>
   <si>
-    <t>van Genuchten model (vb_a, vg_n)</t>
-  </si>
-  <si>
     <t>Unsat model option</t>
-  </si>
-  <si>
-    <t>vg_a</t>
-  </si>
-  <si>
-    <t>vg_n</t>
   </si>
   <si>
     <t>Pore pressure (u) options</t>
@@ -863,6 +815,138 @@
   </si>
   <si>
     <t>Angle</t>
+  </si>
+  <si>
+    <t>Type:</t>
+  </si>
+  <si>
+    <t>Type optons</t>
+  </si>
+  <si>
+    <t>phreatic</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Phreatic surface: static head reduced by cos² of the line's slope.</t>
+  </si>
+  <si>
+    <t>True piezometric line: u = γw × vertical distance below the line (static head).</t>
+  </si>
+  <si>
+    <t>hb</t>
+  </si>
+  <si>
+    <t>gard</t>
+  </si>
+  <si>
+    <t>Gardner model (a, n)</t>
+  </si>
+  <si>
+    <t>van Genuchten model (a, n)</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>hb_sci</t>
+  </si>
+  <si>
+    <t>Generalized Hoek-Brown (rock mass): hb_sci, hb_gsi, hb_mi, hb_d</t>
+  </si>
+  <si>
+    <t>hb_gsi</t>
+  </si>
+  <si>
+    <t>hb_mi</t>
+  </si>
+  <si>
+    <t>hb_d</t>
+  </si>
+  <si>
+    <t>nu</t>
+  </si>
+  <si>
+    <t>BC Option:</t>
+  </si>
+  <si>
+    <t>head</t>
+  </si>
+  <si>
+    <t>flux</t>
+  </si>
+  <si>
+    <t>Head/Flux BC #1</t>
+  </si>
+  <si>
+    <t>specified head (len)</t>
+  </si>
+  <si>
+    <t>Head/Flux BC #2</t>
+  </si>
+  <si>
+    <t>Head/Flux BC #3</t>
+  </si>
+  <si>
+    <t>Head/Flux BC #4</t>
+  </si>
+  <si>
+    <t>Head/Flux BC #5</t>
+  </si>
+  <si>
+    <t>Head/Flux BC #1 (2)</t>
+  </si>
+  <si>
+    <t>Head/Flux BC #2 (2)</t>
+  </si>
+  <si>
+    <t>Head/Flux BC #3 (2)</t>
+  </si>
+  <si>
+    <t>Head/Flux BC #4 (2)</t>
+  </si>
+  <si>
+    <t>Head/Flux BC #5 (2)</t>
+  </si>
+  <si>
+    <t>Neumann flux - normal Darcy velocity (len/time), + = inflow</t>
+  </si>
+  <si>
+    <t>polygon</t>
+  </si>
+  <si>
+    <t>Polygons describing the slope geometry</t>
+  </si>
+  <si>
+    <t>piles</t>
+  </si>
+  <si>
+    <t>Piles</t>
+  </si>
+  <si>
+    <t>lloads</t>
+  </si>
+  <si>
+    <t>Line loads</t>
+  </si>
+  <si>
+    <t>elastic</t>
+  </si>
+  <si>
+    <t>Elastic / infinite strength (cannot fail). FEM: no yield; LEM: impenetrable</t>
+  </si>
+  <si>
+    <t>t_cut</t>
+  </si>
+  <si>
+    <t>Shear Strength/Stiffness</t>
+  </si>
+  <si>
+    <t>Color legend</t>
+  </si>
+  <si>
+    <t>phi_b</t>
+  </si>
+  <si>
+    <t>s_cap</t>
   </si>
 </sst>
 </file>
@@ -1075,12 +1159,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1106,6 +1184,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1196,7 +1280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1253,29 +1337,14 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1294,28 +1363,28 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1328,16 +1397,36 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1345,12 +1434,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1368,14 +1451,14 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="22">
     <dxf>
       <fill>
         <patternFill>
@@ -1394,34 +1477,6 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1463,7 +1518,84 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2560,7 +2692,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>piezo!$A$4:$A$18</c:f>
+              <c:f>piezo!$A$5:$A$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -2569,7 +2701,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>piezo!$B$4:$B$18</c:f>
+              <c:f>piezo!$B$5:$B$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -2621,7 +2753,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>piezo!$D$4:$D$18</c:f>
+              <c:f>piezo!$D$5:$D$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -2630,7 +2762,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>piezo!$E$4:$E$18</c:f>
+              <c:f>piezo!$E$5:$E$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -6141,7 +6273,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Specified Head #1</c:v>
+                  <c:v>Head/Flux BC #1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6210,7 +6342,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Specified Head #2</c:v>
+                  <c:v>Head/Flux BC #2</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6279,7 +6411,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Specified Head #3</c:v>
+                  <c:v>Head/Flux BC #3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6348,7 +6480,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Specified Head #4</c:v>
+                  <c:v>Head/Flux BC #4</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6420,7 +6552,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Specified Head #5</c:v>
+                  <c:v>Head/Flux BC #5</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6564,7 +6696,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Specified Head #1 (2)</c:v>
+                  <c:v>Head/Flux BC #1 (2)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6636,7 +6768,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Specified Head #2 (2)</c:v>
+                  <c:v>Head/Flux BC #2 (2)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6699,7 +6831,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Specified Head #3 (2)</c:v>
+                  <c:v>Head/Flux BC #3 (2)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6762,7 +6894,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Specified Head #4 (2)</c:v>
+                  <c:v>Head/Flux BC #4 (2)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6831,7 +6963,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Specified Head #5 (2)</c:v>
+                  <c:v>Head/Flux BC #5 (2)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -10322,7 +10454,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="19" x14ac:dyDescent="0.25">
@@ -10332,22 +10464,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="35">
-        <v>12</v>
+        <v>78</v>
+      </c>
+      <c r="D5" s="30">
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="49" t="s">
+      <c r="B7" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="36" t="s">
+      <c r="G7" s="31" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10359,10 +10491,10 @@
         <v>9.81</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G8" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -10370,7 +10502,7 @@
         <v>49</v>
       </c>
       <c r="D9" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>19</v>
@@ -10384,7 +10516,7 @@
         <v>48</v>
       </c>
       <c r="D10" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>17</v>
@@ -10396,77 +10528,98 @@
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B11" s="1"/>
       <c r="C11" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D11" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>21</v>
+        <v>227</v>
       </c>
       <c r="G11" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="G13" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F14" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F15" s="1" t="s">
-        <v>118</v>
+        <v>34</v>
       </c>
       <c r="G15" t="s">
-        <v>120</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F16" s="1" t="s">
-        <v>36</v>
+        <v>115</v>
       </c>
       <c r="G16" t="s">
-        <v>37</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>
       <c r="F17" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>122</v>
+        <v>36</v>
+      </c>
+      <c r="G17" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F18" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="G18" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F19" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G19" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F20" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G20" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="G18" s="9" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F21" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="1"/>
@@ -10502,36 +10655,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="61" t="s">
-        <v>142</v>
-      </c>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="F2" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="G2" s="61"/>
-      <c r="H2" s="61"/>
-      <c r="J2" s="61" t="s">
-        <v>144</v>
-      </c>
-      <c r="K2" s="61"/>
-      <c r="L2" s="61"/>
-      <c r="N2" s="61" t="s">
-        <v>145</v>
-      </c>
-      <c r="O2" s="61"/>
-      <c r="P2" s="61"/>
-      <c r="R2" s="61" t="s">
-        <v>146</v>
-      </c>
-      <c r="S2" s="61"/>
-      <c r="T2" s="61"/>
-      <c r="V2" s="61" t="s">
-        <v>147</v>
-      </c>
-      <c r="W2" s="61"/>
-      <c r="X2" s="61"/>
+      <c r="B2" s="60" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="F2" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="J2" s="60" t="s">
+        <v>131</v>
+      </c>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="N2" s="60" t="s">
+        <v>132</v>
+      </c>
+      <c r="O2" s="60"/>
+      <c r="P2" s="60"/>
+      <c r="R2" s="60" t="s">
+        <v>133</v>
+      </c>
+      <c r="S2" s="60"/>
+      <c r="T2" s="60"/>
+      <c r="V2" s="60" t="s">
+        <v>134</v>
+      </c>
+      <c r="W2" s="60"/>
+      <c r="X2" s="60"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -11000,64 +11153,64 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="C2" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="G2" s="40" t="s">
+        <v>192</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>193</v>
+      </c>
+      <c r="I2" s="40" t="s">
+        <v>177</v>
+      </c>
+      <c r="J2" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="K2" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="L2" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="M2" s="27" t="s">
+        <v>178</v>
+      </c>
+      <c r="N2" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="O2" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="P2" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q2" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="R2" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G2" s="45" t="s">
-        <v>208</v>
-      </c>
-      <c r="H2" s="45" t="s">
-        <v>209</v>
-      </c>
-      <c r="I2" s="45" t="s">
-        <v>193</v>
-      </c>
-      <c r="J2" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="K2" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="L2" s="32" t="s">
-        <v>109</v>
-      </c>
-      <c r="M2" s="32" t="s">
-        <v>194</v>
-      </c>
-      <c r="N2" s="32" t="s">
-        <v>195</v>
-      </c>
-      <c r="O2" s="32" t="s">
-        <v>210</v>
-      </c>
-      <c r="P2" s="33" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q2" s="33" t="s">
-        <v>100</v>
-      </c>
-      <c r="R2" s="33" t="s">
-        <v>106</v>
-      </c>
       <c r="Z2" t="s">
-        <v>196</v>
+        <v>180</v>
       </c>
       <c r="AA2" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="AB2" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
@@ -11088,13 +11241,13 @@
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
       <c r="Z3" t="s">
-        <v>199</v>
+        <v>183</v>
       </c>
       <c r="AA3" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="AB3" t="s">
-        <v>201</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.2">
@@ -11125,7 +11278,7 @@
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
       <c r="Z4" t="s">
-        <v>202</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
@@ -11156,7 +11309,7 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="Z5" t="s">
-        <v>203</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -11243,13 +11396,13 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
       <c r="Z8" t="s">
-        <v>196</v>
+        <v>180</v>
       </c>
       <c r="AA8" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="AB8" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
@@ -11280,13 +11433,13 @@
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
       <c r="Z9" t="s">
-        <v>199</v>
+        <v>183</v>
       </c>
       <c r="AA9" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="AB9" t="s">
-        <v>201</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
@@ -11317,13 +11470,13 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
       <c r="Z10" t="s">
-        <v>202</v>
+        <v>186</v>
       </c>
       <c r="AA10" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="AB10" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
@@ -11354,13 +11507,13 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
       <c r="Z11" t="s">
-        <v>203</v>
+        <v>187</v>
       </c>
       <c r="AA11" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="AB11" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
@@ -11672,25 +11825,25 @@
       <c r="R22" s="3"/>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="T23" s="47"/>
+      <c r="T23" s="42"/>
       <c r="U23" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
-      <c r="T24" s="31"/>
+      <c r="T24" s="26"/>
       <c r="U24" s="9" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="K25" s="9"/>
       <c r="L25" s="9"/>
-      <c r="T25" s="34"/>
+      <c r="T25" s="29"/>
       <c r="U25" s="9" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -11728,58 +11881,58 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="C2" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="G2" s="40" t="s">
+        <v>152</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="I2" s="40" t="s">
+        <v>177</v>
+      </c>
+      <c r="J2" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="K2" s="27" t="s">
+        <v>154</v>
+      </c>
+      <c r="L2" s="41" t="s">
+        <v>157</v>
+      </c>
+      <c r="M2" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="N2" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="O2" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="P2" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G2" s="45" t="s">
-        <v>165</v>
-      </c>
-      <c r="H2" s="45" t="s">
-        <v>173</v>
-      </c>
-      <c r="I2" s="45" t="s">
-        <v>193</v>
-      </c>
-      <c r="J2" s="32" t="s">
-        <v>166</v>
-      </c>
-      <c r="K2" s="32" t="s">
-        <v>167</v>
-      </c>
-      <c r="L2" s="46" t="s">
-        <v>170</v>
-      </c>
-      <c r="M2" s="46" t="s">
-        <v>171</v>
-      </c>
-      <c r="N2" s="33" t="s">
-        <v>100</v>
-      </c>
-      <c r="O2" s="33" t="s">
-        <v>168</v>
-      </c>
-      <c r="P2" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q2" s="33" t="s">
-        <v>177</v>
+      <c r="Q2" s="28" t="s">
+        <v>164</v>
       </c>
       <c r="Z2" t="s">
         <v>40</v>
       </c>
       <c r="AA2" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
@@ -11803,10 +11956,10 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="Z3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AA3" t="s">
-        <v>201</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
@@ -12007,21 +12160,21 @@
       <c r="K15" s="9"/>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="S16" s="47"/>
+      <c r="S16" s="42"/>
       <c r="T16" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="19:20" x14ac:dyDescent="0.2">
-      <c r="S17" s="31"/>
+      <c r="S17" s="26"/>
       <c r="T17" s="9" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="19:20" x14ac:dyDescent="0.2">
-      <c r="S18" s="34"/>
+      <c r="S18" s="29"/>
       <c r="T18" s="9" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -12053,7 +12206,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="C2" s="12" t="s">
         <v>3</v>
@@ -12062,10 +12215,10 @@
         <v>4</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>211</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -12275,7 +12428,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D036245-91C1-5842-93DD-735018175DE8}">
-  <dimension ref="B2:R24"/>
+  <dimension ref="B2:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -12286,95 +12439,104 @@
     <col min="16" max="16" width="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="62" t="s">
-        <v>135</v>
-      </c>
-      <c r="C2" s="62"/>
-      <c r="E2" s="58" t="s">
-        <v>130</v>
-      </c>
-      <c r="F2" s="58"/>
-      <c r="H2" s="58" t="s">
-        <v>131</v>
-      </c>
-      <c r="I2" s="58"/>
-      <c r="K2" s="58" t="s">
-        <v>132</v>
-      </c>
-      <c r="L2" s="58"/>
-      <c r="N2" s="58" t="s">
-        <v>133</v>
-      </c>
-      <c r="O2" s="58"/>
-      <c r="Q2" s="58" t="s">
-        <v>134</v>
-      </c>
-      <c r="R2" s="58"/>
-    </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="E3" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="F3" s="38"/>
-      <c r="H3" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="I3" s="38"/>
-      <c r="K3" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="L3" s="38"/>
-      <c r="N3" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="O3" s="38"/>
-      <c r="Q3" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="R3" s="38"/>
-    </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B4" s="28" t="s">
+    <row r="2" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B2" s="61" t="s">
+        <v>127</v>
+      </c>
+      <c r="C2" s="61"/>
+      <c r="E2" s="57" t="s">
+        <v>215</v>
+      </c>
+      <c r="F2" s="57"/>
+      <c r="H2" s="57" t="s">
+        <v>217</v>
+      </c>
+      <c r="I2" s="57"/>
+      <c r="K2" s="57" t="s">
+        <v>218</v>
+      </c>
+      <c r="L2" s="57"/>
+      <c r="N2" s="57" t="s">
+        <v>219</v>
+      </c>
+      <c r="O2" s="57"/>
+      <c r="Q2" s="57" t="s">
+        <v>220</v>
+      </c>
+      <c r="R2" s="57"/>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="E3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="33"/>
+      <c r="H3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="I3" s="33"/>
+      <c r="K3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="L3" s="33"/>
+      <c r="N3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="O3" s="33"/>
+      <c r="Q3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="R3" s="33"/>
+      <c r="T3" s="6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="28" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="28" t="s">
+      <c r="H4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="28" t="s">
+      <c r="I4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="28" t="s">
+      <c r="K4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="L4" s="28" t="s">
+      <c r="L4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="28" t="s">
+      <c r="N4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="O4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="Q4" s="28" t="s">
+      <c r="Q4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="R4" s="28" t="s">
+      <c r="R4" s="25" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="T4" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="U4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" s="3"/>
@@ -12387,8 +12549,14 @@
       <c r="O5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-    </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="T5" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="U5" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="6" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="E6" s="3"/>
@@ -12401,8 +12569,10 @@
       <c r="O6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
-    </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="T6" s="1"/>
+      <c r="U6" s="9"/>
+    </row>
+    <row r="7" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="E7" s="3"/>
@@ -12416,7 +12586,7 @@
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="E8" s="3"/>
@@ -12430,7 +12600,7 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
     </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="E9" s="3"/>
@@ -12444,7 +12614,7 @@
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="E10" s="3"/>
@@ -12458,7 +12628,7 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
     </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="E11" s="3"/>
@@ -12472,7 +12642,7 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="E12" s="3"/>
@@ -12486,7 +12656,7 @@
       <c r="Q12" s="3"/>
       <c r="R12" s="3"/>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="E13" s="3"/>
@@ -12500,7 +12670,7 @@
       <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
     </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="E14" s="3"/>
@@ -12514,7 +12684,7 @@
       <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
     </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="E15" s="3"/>
@@ -12528,7 +12698,7 @@
       <c r="Q15" s="3"/>
       <c r="R15" s="3"/>
     </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="E16" s="3"/>
@@ -12663,13 +12833,18 @@
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3 H3 K3 N3 Q3" xr:uid="{21F200C9-4829-4345-9958-0F754F272AD0}">
+      <formula1>$T$4:$T$5</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C3C734-6227-7445-884D-1F1A5F3909C7}">
-  <dimension ref="B2:R24"/>
+  <dimension ref="B2:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -12680,95 +12855,104 @@
     <col min="16" max="16" width="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="63" t="s">
-        <v>137</v>
-      </c>
-      <c r="C2" s="63"/>
-      <c r="E2" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="F2" s="59"/>
-      <c r="H2" s="59" t="s">
-        <v>138</v>
-      </c>
-      <c r="I2" s="59"/>
-      <c r="K2" s="59" t="s">
-        <v>139</v>
-      </c>
-      <c r="L2" s="59"/>
-      <c r="N2" s="59" t="s">
-        <v>140</v>
-      </c>
-      <c r="O2" s="59"/>
-      <c r="Q2" s="59" t="s">
-        <v>141</v>
-      </c>
-      <c r="R2" s="59"/>
-    </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="E3" s="39" t="s">
-        <v>94</v>
-      </c>
-      <c r="F3" s="40"/>
-      <c r="H3" s="39" t="s">
-        <v>94</v>
-      </c>
-      <c r="I3" s="40"/>
-      <c r="K3" s="39" t="s">
-        <v>94</v>
-      </c>
-      <c r="L3" s="40"/>
-      <c r="N3" s="39" t="s">
-        <v>94</v>
-      </c>
-      <c r="O3" s="40"/>
-      <c r="Q3" s="39" t="s">
-        <v>94</v>
-      </c>
-      <c r="R3" s="40"/>
-    </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B4" s="28" t="s">
+    <row r="2" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B2" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="C2" s="62"/>
+      <c r="E2" s="58" t="s">
+        <v>221</v>
+      </c>
+      <c r="F2" s="58"/>
+      <c r="H2" s="58" t="s">
+        <v>222</v>
+      </c>
+      <c r="I2" s="58"/>
+      <c r="K2" s="58" t="s">
+        <v>223</v>
+      </c>
+      <c r="L2" s="58"/>
+      <c r="N2" s="58" t="s">
+        <v>224</v>
+      </c>
+      <c r="O2" s="58"/>
+      <c r="Q2" s="58" t="s">
+        <v>225</v>
+      </c>
+      <c r="R2" s="58"/>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="E3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="35"/>
+      <c r="H3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="I3" s="35"/>
+      <c r="K3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="L3" s="35"/>
+      <c r="N3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="O3" s="35"/>
+      <c r="Q3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="R3" s="35"/>
+      <c r="T3" s="6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="28" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="28" t="s">
+      <c r="H4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="28" t="s">
+      <c r="I4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="28" t="s">
+      <c r="K4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="L4" s="28" t="s">
+      <c r="L4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="28" t="s">
+      <c r="N4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="O4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="Q4" s="28" t="s">
+      <c r="Q4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="R4" s="28" t="s">
+      <c r="R4" s="25" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="T4" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="U4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" s="3"/>
@@ -12781,8 +12965,14 @@
       <c r="O5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-    </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="T5" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="U5" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="6" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="E6" s="3"/>
@@ -12796,7 +12986,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="E7" s="3"/>
@@ -12810,7 +13000,7 @@
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="E8" s="3"/>
@@ -12824,7 +13014,7 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
     </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="E9" s="3"/>
@@ -12838,7 +13028,7 @@
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="E10" s="3"/>
@@ -12852,7 +13042,7 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
     </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="E11" s="3"/>
@@ -12866,7 +13056,7 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="E12" s="3"/>
@@ -12880,7 +13070,7 @@
       <c r="Q12" s="3"/>
       <c r="R12" s="3"/>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="E13" s="3"/>
@@ -12894,7 +13084,7 @@
       <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
     </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="E14" s="3"/>
@@ -12908,7 +13098,7 @@
       <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
     </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="E15" s="3"/>
@@ -12922,7 +13112,7 @@
       <c r="Q15" s="3"/>
       <c r="R15" s="3"/>
     </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="E16" s="3"/>
@@ -13057,6 +13247,11 @@
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="N2:O2"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3 H3 K3 N3 Q3" xr:uid="{68C61D93-1721-F843-8E53-0F0E50006C65}">
+      <formula1>$T$4:$T$5</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -13073,364 +13268,346 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A900FC-A692-B445-95C9-59E70352B291}">
-  <dimension ref="A2:AG51"/>
+  <dimension ref="A2:AN52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="31" width="8.5" customWidth="1"/>
-    <col min="32" max="32" width="8.5" style="1" customWidth="1"/>
-    <col min="33" max="33" width="8.5" customWidth="1"/>
+    <col min="11" max="40" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2"/>
-      <c r="K2" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="U2" s="6"/>
-      <c r="AA2" s="6" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="L2" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="AD2" s="6"/>
+      <c r="AJ2" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F3"/>
       <c r="G3"/>
-      <c r="K3" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="L3" t="s">
-        <v>59</v>
-      </c>
-      <c r="U3" s="14"/>
-      <c r="AA3" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="O3" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="P3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD3" s="14"/>
+      <c r="AJ3" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" t="s">
         <v>70</v>
-      </c>
-      <c r="D4" t="s">
-        <v>71</v>
       </c>
       <c r="F4"/>
       <c r="G4"/>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="42"/>
+      <c r="M4" t="s">
+        <v>161</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="L4" t="s">
-        <v>60</v>
-      </c>
-      <c r="U4" s="14"/>
-      <c r="AA4" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="P4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AD4" s="14"/>
+      <c r="AJ4" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C5" s="1" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="D5" t="s">
+        <v>191</v>
+      </c>
+      <c r="L5" s="26"/>
+      <c r="M5" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="P5" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD5" s="14"/>
+      <c r="AJ5" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="AK5" s="9" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="6" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="C6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L6" s="29"/>
+      <c r="M6" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="P6" t="s">
+        <v>190</v>
+      </c>
+      <c r="AE6" s="1"/>
+      <c r="AF6" s="1"/>
+    </row>
+    <row r="7" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="C7" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="AE7" s="1"/>
+      <c r="AF7" s="1"/>
+    </row>
+    <row r="9" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="C9" s="51" t="s">
+        <v>236</v>
+      </c>
+      <c r="D9" s="51"/>
+      <c r="E9" s="51"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="51"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="51"/>
+      <c r="O9" s="51"/>
+      <c r="P9" s="51"/>
+      <c r="Q9" s="51"/>
+      <c r="R9" s="51"/>
+      <c r="S9" s="51"/>
+      <c r="T9" s="51"/>
+      <c r="U9" s="51"/>
+      <c r="V9" s="51"/>
+      <c r="W9" s="51"/>
+      <c r="X9" s="51"/>
+      <c r="Y9" s="51"/>
+      <c r="Z9" s="51"/>
+      <c r="AA9" s="51" t="s">
+        <v>57</v>
+      </c>
+      <c r="AB9" s="51"/>
+      <c r="AC9" s="51"/>
+      <c r="AD9" s="51"/>
+      <c r="AE9" s="51"/>
+      <c r="AF9" s="51"/>
+      <c r="AG9" s="51" t="s">
+        <v>91</v>
+      </c>
+      <c r="AH9" s="51"/>
+      <c r="AI9" s="51"/>
+      <c r="AJ9" s="51"/>
+      <c r="AK9" s="51"/>
+      <c r="AL9" s="51"/>
+      <c r="AM9" s="51"/>
+      <c r="AN9" s="51"/>
+    </row>
+    <row r="10" spans="1:40" ht="18" x14ac:dyDescent="0.25">
+      <c r="A10" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="45" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="48" t="s">
+        <v>189</v>
+      </c>
+      <c r="E10" s="44" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" s="44" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" s="44" t="s">
+        <v>71</v>
+      </c>
+      <c r="J10" s="49" t="s">
+        <v>79</v>
+      </c>
+      <c r="K10" s="49" t="s">
+        <v>135</v>
+      </c>
+      <c r="L10" s="21" t="s">
+        <v>235</v>
+      </c>
+      <c r="M10" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="N10" s="43" t="s">
+        <v>211</v>
+      </c>
+      <c r="O10" s="44" t="s">
+        <v>84</v>
+      </c>
+      <c r="P10" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q10" s="44" t="s">
+        <v>238</v>
+      </c>
+      <c r="R10" s="44" t="s">
+        <v>239</v>
+      </c>
+      <c r="S10" s="44" t="s">
+        <v>173</v>
+      </c>
+      <c r="T10" s="44" t="s">
+        <v>174</v>
+      </c>
+      <c r="U10" s="44" t="s">
+        <v>175</v>
+      </c>
+      <c r="V10" s="44" t="s">
+        <v>176</v>
+      </c>
+      <c r="W10" s="44" t="s">
+        <v>206</v>
+      </c>
+      <c r="X10" s="44" t="s">
+        <v>208</v>
+      </c>
+      <c r="Y10" s="44" t="s">
+        <v>209</v>
+      </c>
+      <c r="Z10" s="44" t="s">
+        <v>210</v>
+      </c>
+      <c r="AA10" s="46" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB10" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="AC10" s="47" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD10" s="46" t="s">
+        <v>73</v>
+      </c>
+      <c r="AE10" s="46" t="s">
+        <v>80</v>
+      </c>
+      <c r="AF10" s="47" t="s">
+        <v>136</v>
+      </c>
+      <c r="AG10" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="L5" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="U5" s="14"/>
-      <c r="AA5" s="1"/>
-      <c r="AB5" s="9"/>
-    </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.2">
-      <c r="K6" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="L6" t="s">
-        <v>206</v>
-      </c>
-      <c r="P6" s="1"/>
-      <c r="V6" s="1"/>
-      <c r="W6" s="1"/>
-    </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.2">
-      <c r="C8" s="50" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" s="51"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="50"/>
-      <c r="G8" s="50"/>
-      <c r="H8" s="50"/>
-      <c r="I8" s="50"/>
-      <c r="J8" s="50"/>
-      <c r="K8" s="50"/>
-      <c r="L8" s="52"/>
-      <c r="M8" s="52"/>
-      <c r="N8" s="52"/>
-      <c r="O8" s="52"/>
-      <c r="P8" s="1"/>
-      <c r="R8" s="50" t="s">
-        <v>58</v>
-      </c>
-      <c r="S8" s="50"/>
-      <c r="T8" s="50"/>
-      <c r="U8" s="50"/>
-      <c r="V8" s="50"/>
-      <c r="W8" s="50"/>
-      <c r="X8" s="50" t="s">
-        <v>92</v>
-      </c>
-      <c r="Y8" s="50"/>
-      <c r="Z8" s="50"/>
-      <c r="AA8" s="50"/>
-      <c r="AB8" s="50"/>
-      <c r="AC8" s="50"/>
-      <c r="AD8" s="50"/>
-      <c r="AE8" s="50"/>
-      <c r="AF8" s="50" t="s">
-        <v>99</v>
-      </c>
-      <c r="AG8" s="50"/>
-    </row>
-    <row r="9" spans="1:33" ht="18" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="48" t="s">
+      <c r="AH10" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="AI10" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="AJ10" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK10" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="AL10" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM10" s="23" t="s">
         <v>205</v>
       </c>
-      <c r="E9" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="H9" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="I9" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="J9" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="K9" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="L9" s="21" t="s">
-        <v>189</v>
-      </c>
-      <c r="M9" s="21" t="s">
-        <v>190</v>
-      </c>
-      <c r="N9" s="21" t="s">
-        <v>191</v>
-      </c>
-      <c r="O9" s="21" t="s">
-        <v>192</v>
-      </c>
-      <c r="P9" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q9" s="21" t="s">
-        <v>188</v>
-      </c>
-      <c r="R9" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="S9" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="T9" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="U9" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="V9" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="W9" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="X9" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y9" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z9" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA9" s="25" t="s">
-        <v>178</v>
-      </c>
-      <c r="AB9" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="AC9" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="AD9" s="25" t="s">
-        <v>184</v>
-      </c>
-      <c r="AE9" s="25" t="s">
-        <v>185</v>
-      </c>
-      <c r="AF9" s="29" t="s">
-        <v>100</v>
-      </c>
-      <c r="AG9" s="30" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
+      <c r="AN10" s="23" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
         <v>1</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Embankment</t>
         </is>
       </c>
-      <c r="C10" s="3">
+      <c r="C11" s="3">
         <v>18.2</v>
       </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="D11" s="3"/>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
-      <c r="F10" s="3">
+      <c r="F11" s="3">
         <v>13.8</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G11" s="3">
         <v>37.0</v>
       </c>
-      <c r="H10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="I10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="J10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="K10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Q10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="R10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="S10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="T10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="U10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="V10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="W10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="X10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="Y10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="Z10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="AA10" s="3" t="inlineStr">
-        <is>
-          <t>lf</t>
-        </is>
-      </c>
-      <c r="AB10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="AC10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="AD10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="AE10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="AF10" s="3">
-        <v>100000.0</v>
-      </c>
-      <c r="AG10" s="3">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
-        <v>2</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
+      <c r="M11" s="3">
+        <v>100000.0</v>
+      </c>
+      <c r="N11" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
@@ -13445,14 +13622,21 @@
       <c r="AA11" s="3"/>
       <c r="AB11" s="3"/>
       <c r="AC11" s="3"/>
-      <c r="AD11" s="18"/>
-      <c r="AE11" s="19"/>
+      <c r="AD11" s="3"/>
+      <c r="AE11" s="3"/>
       <c r="AF11" s="3"/>
       <c r="AG11" s="3"/>
-    </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH11" s="3"/>
+      <c r="AI11" s="3"/>
+      <c r="AJ11" s="3"/>
+      <c r="AK11" s="3"/>
+      <c r="AL11" s="3"/>
+      <c r="AM11" s="3"/>
+      <c r="AN11" s="3"/>
+    </row>
+    <row r="12" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -13482,14 +13666,21 @@
       <c r="AA12" s="3"/>
       <c r="AB12" s="3"/>
       <c r="AC12" s="3"/>
-      <c r="AD12" s="18"/>
-      <c r="AE12" s="19"/>
+      <c r="AD12" s="3"/>
+      <c r="AE12" s="3"/>
       <c r="AF12" s="3"/>
       <c r="AG12" s="3"/>
-    </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH12" s="3"/>
+      <c r="AI12" s="3"/>
+      <c r="AJ12" s="3"/>
+      <c r="AK12" s="3"/>
+      <c r="AL12" s="3"/>
+      <c r="AM12" s="18"/>
+      <c r="AN12" s="19"/>
+    </row>
+    <row r="13" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -13523,10 +13714,17 @@
       <c r="AE13" s="3"/>
       <c r="AF13" s="3"/>
       <c r="AG13" s="3"/>
-    </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH13" s="3"/>
+      <c r="AI13" s="3"/>
+      <c r="AJ13" s="3"/>
+      <c r="AK13" s="3"/>
+      <c r="AL13" s="3"/>
+      <c r="AM13" s="18"/>
+      <c r="AN13" s="19"/>
+    </row>
+    <row r="14" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -13560,10 +13758,17 @@
       <c r="AE14" s="3"/>
       <c r="AF14" s="3"/>
       <c r="AG14" s="3"/>
-    </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH14" s="3"/>
+      <c r="AI14" s="3"/>
+      <c r="AJ14" s="3"/>
+      <c r="AK14" s="3"/>
+      <c r="AL14" s="3"/>
+      <c r="AM14" s="3"/>
+      <c r="AN14" s="3"/>
+    </row>
+    <row r="15" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -13597,10 +13802,17 @@
       <c r="AE15" s="3"/>
       <c r="AF15" s="3"/>
       <c r="AG15" s="3"/>
-    </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH15" s="3"/>
+      <c r="AI15" s="3"/>
+      <c r="AJ15" s="3"/>
+      <c r="AK15" s="3"/>
+      <c r="AL15" s="3"/>
+      <c r="AM15" s="3"/>
+      <c r="AN15" s="3"/>
+    </row>
+    <row r="16" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -13634,10 +13846,17 @@
       <c r="AE16" s="3"/>
       <c r="AF16" s="3"/>
       <c r="AG16" s="3"/>
-    </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH16" s="3"/>
+      <c r="AI16" s="3"/>
+      <c r="AJ16" s="3"/>
+      <c r="AK16" s="3"/>
+      <c r="AL16" s="3"/>
+      <c r="AM16" s="3"/>
+      <c r="AN16" s="3"/>
+    </row>
+    <row r="17" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -13671,10 +13890,17 @@
       <c r="AE17" s="3"/>
       <c r="AF17" s="3"/>
       <c r="AG17" s="3"/>
-    </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH17" s="3"/>
+      <c r="AI17" s="3"/>
+      <c r="AJ17" s="3"/>
+      <c r="AK17" s="3"/>
+      <c r="AL17" s="3"/>
+      <c r="AM17" s="3"/>
+      <c r="AN17" s="3"/>
+    </row>
+    <row r="18" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -13708,10 +13934,17 @@
       <c r="AE18" s="3"/>
       <c r="AF18" s="3"/>
       <c r="AG18" s="3"/>
-    </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH18" s="3"/>
+      <c r="AI18" s="3"/>
+      <c r="AJ18" s="3"/>
+      <c r="AK18" s="3"/>
+      <c r="AL18" s="3"/>
+      <c r="AM18" s="3"/>
+      <c r="AN18" s="3"/>
+    </row>
+    <row r="19" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -13745,10 +13978,17 @@
       <c r="AE19" s="3"/>
       <c r="AF19" s="3"/>
       <c r="AG19" s="3"/>
-    </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH19" s="3"/>
+      <c r="AI19" s="3"/>
+      <c r="AJ19" s="3"/>
+      <c r="AK19" s="3"/>
+      <c r="AL19" s="3"/>
+      <c r="AM19" s="3"/>
+      <c r="AN19" s="3"/>
+    </row>
+    <row r="20" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -13782,10 +14022,17 @@
       <c r="AE20" s="3"/>
       <c r="AF20" s="3"/>
       <c r="AG20" s="3"/>
-    </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH20" s="3"/>
+      <c r="AI20" s="3"/>
+      <c r="AJ20" s="3"/>
+      <c r="AK20" s="3"/>
+      <c r="AL20" s="3"/>
+      <c r="AM20" s="3"/>
+      <c r="AN20" s="3"/>
+    </row>
+    <row r="21" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -13819,10 +14066,17 @@
       <c r="AE21" s="3"/>
       <c r="AF21" s="3"/>
       <c r="AG21" s="3"/>
-    </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH21" s="3"/>
+      <c r="AI21" s="3"/>
+      <c r="AJ21" s="3"/>
+      <c r="AK21" s="3"/>
+      <c r="AL21" s="3"/>
+      <c r="AM21" s="3"/>
+      <c r="AN21" s="3"/>
+    </row>
+    <row r="22" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -13856,10 +14110,17 @@
       <c r="AE22" s="3"/>
       <c r="AF22" s="3"/>
       <c r="AG22" s="3"/>
-    </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH22" s="3"/>
+      <c r="AI22" s="3"/>
+      <c r="AJ22" s="3"/>
+      <c r="AK22" s="3"/>
+      <c r="AL22" s="3"/>
+      <c r="AM22" s="3"/>
+      <c r="AN22" s="3"/>
+    </row>
+    <row r="23" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -13893,10 +14154,17 @@
       <c r="AE23" s="3"/>
       <c r="AF23" s="3"/>
       <c r="AG23" s="3"/>
-    </row>
-    <row r="24" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH23" s="3"/>
+      <c r="AI23" s="3"/>
+      <c r="AJ23" s="3"/>
+      <c r="AK23" s="3"/>
+      <c r="AL23" s="3"/>
+      <c r="AM23" s="3"/>
+      <c r="AN23" s="3"/>
+    </row>
+    <row r="24" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -13930,31 +14198,59 @@
       <c r="AE24" s="3"/>
       <c r="AF24" s="3"/>
       <c r="AG24" s="3"/>
-    </row>
-    <row r="25" spans="1:33" x14ac:dyDescent="0.2">
-      <c r="K25" s="1"/>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
-      <c r="Q25" s="1"/>
-      <c r="R25" s="1"/>
-      <c r="S25" s="1"/>
-      <c r="T25" s="1"/>
-      <c r="U25" s="1"/>
-      <c r="V25" s="1"/>
-      <c r="W25" s="1"/>
-      <c r="X25" s="1"/>
-      <c r="Y25" s="1"/>
-      <c r="Z25" s="1"/>
-      <c r="AA25" s="1"/>
-      <c r="AB25" s="1"/>
-      <c r="AC25" s="1"/>
-      <c r="AD25" s="1"/>
-      <c r="AE25" s="1"/>
-    </row>
-    <row r="26" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="AH24" s="3"/>
+      <c r="AI24" s="3"/>
+      <c r="AJ24" s="3"/>
+      <c r="AK24" s="3"/>
+      <c r="AL24" s="3"/>
+      <c r="AM24" s="3"/>
+      <c r="AN24" s="3"/>
+    </row>
+    <row r="25" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>15</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="3"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="3"/>
+      <c r="X25" s="3"/>
+      <c r="Y25" s="3"/>
+      <c r="Z25" s="3"/>
+      <c r="AA25" s="3"/>
+      <c r="AB25" s="3"/>
+      <c r="AC25" s="3"/>
+      <c r="AD25" s="3"/>
+      <c r="AE25" s="3"/>
+      <c r="AF25" s="3"/>
+      <c r="AG25" s="3"/>
+      <c r="AH25" s="3"/>
+      <c r="AI25" s="3"/>
+      <c r="AJ25" s="3"/>
+      <c r="AK25" s="3"/>
+      <c r="AL25" s="3"/>
+      <c r="AM25" s="3"/>
+      <c r="AN25" s="3"/>
+    </row>
+    <row r="26" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -13968,8 +14264,25 @@
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
       <c r="W26" s="1"/>
-    </row>
-    <row r="27" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="X26" s="1"/>
+      <c r="Y26" s="1"/>
+      <c r="Z26" s="1"/>
+      <c r="AA26" s="1"/>
+      <c r="AB26" s="1"/>
+      <c r="AC26" s="1"/>
+      <c r="AD26" s="1"/>
+      <c r="AE26" s="1"/>
+      <c r="AF26" s="1"/>
+      <c r="AG26" s="1"/>
+      <c r="AH26" s="1"/>
+      <c r="AI26" s="1"/>
+      <c r="AJ26" s="1"/>
+      <c r="AK26" s="1"/>
+      <c r="AL26" s="1"/>
+      <c r="AM26" s="1"/>
+      <c r="AN26" s="1"/>
+    </row>
+    <row r="27" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -13983,8 +14296,17 @@
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
       <c r="W27" s="1"/>
-    </row>
-    <row r="28" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="X27" s="1"/>
+      <c r="Y27" s="1"/>
+      <c r="Z27" s="1"/>
+      <c r="AA27" s="1"/>
+      <c r="AB27" s="1"/>
+      <c r="AC27" s="1"/>
+      <c r="AD27" s="1"/>
+      <c r="AE27" s="1"/>
+      <c r="AF27" s="1"/>
+    </row>
+    <row r="28" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -13998,8 +14320,17 @@
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
       <c r="W28" s="1"/>
-    </row>
-    <row r="29" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="X28" s="1"/>
+      <c r="Y28" s="1"/>
+      <c r="Z28" s="1"/>
+      <c r="AA28" s="1"/>
+      <c r="AB28" s="1"/>
+      <c r="AC28" s="1"/>
+      <c r="AD28" s="1"/>
+      <c r="AE28" s="1"/>
+      <c r="AF28" s="1"/>
+    </row>
+    <row r="29" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -14013,8 +14344,17 @@
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
       <c r="W29" s="1"/>
-    </row>
-    <row r="30" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="X29" s="1"/>
+      <c r="Y29" s="1"/>
+      <c r="Z29" s="1"/>
+      <c r="AA29" s="1"/>
+      <c r="AB29" s="1"/>
+      <c r="AC29" s="1"/>
+      <c r="AD29" s="1"/>
+      <c r="AE29" s="1"/>
+      <c r="AF29" s="1"/>
+    </row>
+    <row r="30" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -14028,8 +14368,17 @@
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
       <c r="W30" s="1"/>
-    </row>
-    <row r="31" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="X30" s="1"/>
+      <c r="Y30" s="1"/>
+      <c r="Z30" s="1"/>
+      <c r="AA30" s="1"/>
+      <c r="AB30" s="1"/>
+      <c r="AC30" s="1"/>
+      <c r="AD30" s="1"/>
+      <c r="AE30" s="1"/>
+      <c r="AF30" s="1"/>
+    </row>
+    <row r="31" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -14043,8 +14392,17 @@
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
       <c r="W31" s="1"/>
-    </row>
-    <row r="32" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="X31" s="1"/>
+      <c r="Y31" s="1"/>
+      <c r="Z31" s="1"/>
+      <c r="AA31" s="1"/>
+      <c r="AB31" s="1"/>
+      <c r="AC31" s="1"/>
+      <c r="AD31" s="1"/>
+      <c r="AE31" s="1"/>
+      <c r="AF31" s="1"/>
+    </row>
+    <row r="32" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -14058,8 +14416,17 @@
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
-    </row>
-    <row r="33" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X32" s="1"/>
+      <c r="Y32" s="1"/>
+      <c r="Z32" s="1"/>
+      <c r="AA32" s="1"/>
+      <c r="AB32" s="1"/>
+      <c r="AC32" s="1"/>
+      <c r="AD32" s="1"/>
+      <c r="AE32" s="1"/>
+      <c r="AF32" s="1"/>
+    </row>
+    <row r="33" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -14073,8 +14440,17 @@
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
       <c r="W33" s="1"/>
-    </row>
-    <row r="34" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X33" s="1"/>
+      <c r="Y33" s="1"/>
+      <c r="Z33" s="1"/>
+      <c r="AA33" s="1"/>
+      <c r="AB33" s="1"/>
+      <c r="AC33" s="1"/>
+      <c r="AD33" s="1"/>
+      <c r="AE33" s="1"/>
+      <c r="AF33" s="1"/>
+    </row>
+    <row r="34" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -14088,8 +14464,17 @@
       <c r="U34" s="1"/>
       <c r="V34" s="1"/>
       <c r="W34" s="1"/>
-    </row>
-    <row r="35" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X34" s="1"/>
+      <c r="Y34" s="1"/>
+      <c r="Z34" s="1"/>
+      <c r="AA34" s="1"/>
+      <c r="AB34" s="1"/>
+      <c r="AC34" s="1"/>
+      <c r="AD34" s="1"/>
+      <c r="AE34" s="1"/>
+      <c r="AF34" s="1"/>
+    </row>
+    <row r="35" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
@@ -14103,8 +14488,17 @@
       <c r="U35" s="1"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
-    </row>
-    <row r="36" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X35" s="1"/>
+      <c r="Y35" s="1"/>
+      <c r="Z35" s="1"/>
+      <c r="AA35" s="1"/>
+      <c r="AB35" s="1"/>
+      <c r="AC35" s="1"/>
+      <c r="AD35" s="1"/>
+      <c r="AE35" s="1"/>
+      <c r="AF35" s="1"/>
+    </row>
+    <row r="36" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -14118,8 +14512,17 @@
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
       <c r="W36" s="1"/>
-    </row>
-    <row r="37" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X36" s="1"/>
+      <c r="Y36" s="1"/>
+      <c r="Z36" s="1"/>
+      <c r="AA36" s="1"/>
+      <c r="AB36" s="1"/>
+      <c r="AC36" s="1"/>
+      <c r="AD36" s="1"/>
+      <c r="AE36" s="1"/>
+      <c r="AF36" s="1"/>
+    </row>
+    <row r="37" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -14133,8 +14536,17 @@
       <c r="U37" s="1"/>
       <c r="V37" s="1"/>
       <c r="W37" s="1"/>
-    </row>
-    <row r="38" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X37" s="1"/>
+      <c r="Y37" s="1"/>
+      <c r="Z37" s="1"/>
+      <c r="AA37" s="1"/>
+      <c r="AB37" s="1"/>
+      <c r="AC37" s="1"/>
+      <c r="AD37" s="1"/>
+      <c r="AE37" s="1"/>
+      <c r="AF37" s="1"/>
+    </row>
+    <row r="38" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
@@ -14148,8 +14560,17 @@
       <c r="U38" s="1"/>
       <c r="V38" s="1"/>
       <c r="W38" s="1"/>
-    </row>
-    <row r="39" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X38" s="1"/>
+      <c r="Y38" s="1"/>
+      <c r="Z38" s="1"/>
+      <c r="AA38" s="1"/>
+      <c r="AB38" s="1"/>
+      <c r="AC38" s="1"/>
+      <c r="AD38" s="1"/>
+      <c r="AE38" s="1"/>
+      <c r="AF38" s="1"/>
+    </row>
+    <row r="39" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -14163,8 +14584,17 @@
       <c r="U39" s="1"/>
       <c r="V39" s="1"/>
       <c r="W39" s="1"/>
-    </row>
-    <row r="40" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X39" s="1"/>
+      <c r="Y39" s="1"/>
+      <c r="Z39" s="1"/>
+      <c r="AA39" s="1"/>
+      <c r="AB39" s="1"/>
+      <c r="AC39" s="1"/>
+      <c r="AD39" s="1"/>
+      <c r="AE39" s="1"/>
+      <c r="AF39" s="1"/>
+    </row>
+    <row r="40" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -14178,8 +14608,17 @@
       <c r="U40" s="1"/>
       <c r="V40" s="1"/>
       <c r="W40" s="1"/>
-    </row>
-    <row r="41" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X40" s="1"/>
+      <c r="Y40" s="1"/>
+      <c r="Z40" s="1"/>
+      <c r="AA40" s="1"/>
+      <c r="AB40" s="1"/>
+      <c r="AC40" s="1"/>
+      <c r="AD40" s="1"/>
+      <c r="AE40" s="1"/>
+      <c r="AF40" s="1"/>
+    </row>
+    <row r="41" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
@@ -14193,8 +14632,17 @@
       <c r="U41" s="1"/>
       <c r="V41" s="1"/>
       <c r="W41" s="1"/>
-    </row>
-    <row r="42" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X41" s="1"/>
+      <c r="Y41" s="1"/>
+      <c r="Z41" s="1"/>
+      <c r="AA41" s="1"/>
+      <c r="AB41" s="1"/>
+      <c r="AC41" s="1"/>
+      <c r="AD41" s="1"/>
+      <c r="AE41" s="1"/>
+      <c r="AF41" s="1"/>
+    </row>
+    <row r="42" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
@@ -14208,8 +14656,17 @@
       <c r="U42" s="1"/>
       <c r="V42" s="1"/>
       <c r="W42" s="1"/>
-    </row>
-    <row r="43" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X42" s="1"/>
+      <c r="Y42" s="1"/>
+      <c r="Z42" s="1"/>
+      <c r="AA42" s="1"/>
+      <c r="AB42" s="1"/>
+      <c r="AC42" s="1"/>
+      <c r="AD42" s="1"/>
+      <c r="AE42" s="1"/>
+      <c r="AF42" s="1"/>
+    </row>
+    <row r="43" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
@@ -14223,8 +14680,17 @@
       <c r="U43" s="1"/>
       <c r="V43" s="1"/>
       <c r="W43" s="1"/>
-    </row>
-    <row r="44" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X43" s="1"/>
+      <c r="Y43" s="1"/>
+      <c r="Z43" s="1"/>
+      <c r="AA43" s="1"/>
+      <c r="AB43" s="1"/>
+      <c r="AC43" s="1"/>
+      <c r="AD43" s="1"/>
+      <c r="AE43" s="1"/>
+      <c r="AF43" s="1"/>
+    </row>
+    <row r="44" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
@@ -14238,8 +14704,17 @@
       <c r="U44" s="1"/>
       <c r="V44" s="1"/>
       <c r="W44" s="1"/>
-    </row>
-    <row r="45" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X44" s="1"/>
+      <c r="Y44" s="1"/>
+      <c r="Z44" s="1"/>
+      <c r="AA44" s="1"/>
+      <c r="AB44" s="1"/>
+      <c r="AC44" s="1"/>
+      <c r="AD44" s="1"/>
+      <c r="AE44" s="1"/>
+      <c r="AF44" s="1"/>
+    </row>
+    <row r="45" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
@@ -14253,8 +14728,17 @@
       <c r="U45" s="1"/>
       <c r="V45" s="1"/>
       <c r="W45" s="1"/>
-    </row>
-    <row r="46" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X45" s="1"/>
+      <c r="Y45" s="1"/>
+      <c r="Z45" s="1"/>
+      <c r="AA45" s="1"/>
+      <c r="AB45" s="1"/>
+      <c r="AC45" s="1"/>
+      <c r="AD45" s="1"/>
+      <c r="AE45" s="1"/>
+      <c r="AF45" s="1"/>
+    </row>
+    <row r="46" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
@@ -14268,8 +14752,17 @@
       <c r="U46" s="1"/>
       <c r="V46" s="1"/>
       <c r="W46" s="1"/>
-    </row>
-    <row r="47" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X46" s="1"/>
+      <c r="Y46" s="1"/>
+      <c r="Z46" s="1"/>
+      <c r="AA46" s="1"/>
+      <c r="AB46" s="1"/>
+      <c r="AC46" s="1"/>
+      <c r="AD46" s="1"/>
+      <c r="AE46" s="1"/>
+      <c r="AF46" s="1"/>
+    </row>
+    <row r="47" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
@@ -14283,8 +14776,17 @@
       <c r="U47" s="1"/>
       <c r="V47" s="1"/>
       <c r="W47" s="1"/>
-    </row>
-    <row r="48" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X47" s="1"/>
+      <c r="Y47" s="1"/>
+      <c r="Z47" s="1"/>
+      <c r="AA47" s="1"/>
+      <c r="AB47" s="1"/>
+      <c r="AC47" s="1"/>
+      <c r="AD47" s="1"/>
+      <c r="AE47" s="1"/>
+      <c r="AF47" s="1"/>
+    </row>
+    <row r="48" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
@@ -14298,8 +14800,17 @@
       <c r="U48" s="1"/>
       <c r="V48" s="1"/>
       <c r="W48" s="1"/>
-    </row>
-    <row r="49" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X48" s="1"/>
+      <c r="Y48" s="1"/>
+      <c r="Z48" s="1"/>
+      <c r="AA48" s="1"/>
+      <c r="AB48" s="1"/>
+      <c r="AC48" s="1"/>
+      <c r="AD48" s="1"/>
+      <c r="AE48" s="1"/>
+      <c r="AF48" s="1"/>
+    </row>
+    <row r="49" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
@@ -14313,8 +14824,17 @@
       <c r="U49" s="1"/>
       <c r="V49" s="1"/>
       <c r="W49" s="1"/>
-    </row>
-    <row r="50" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X49" s="1"/>
+      <c r="Y49" s="1"/>
+      <c r="Z49" s="1"/>
+      <c r="AA49" s="1"/>
+      <c r="AB49" s="1"/>
+      <c r="AC49" s="1"/>
+      <c r="AD49" s="1"/>
+      <c r="AE49" s="1"/>
+      <c r="AF49" s="1"/>
+    </row>
+    <row r="50" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
@@ -14328,8 +14848,17 @@
       <c r="U50" s="1"/>
       <c r="V50" s="1"/>
       <c r="W50" s="1"/>
-    </row>
-    <row r="51" spans="11:23" x14ac:dyDescent="0.2">
+      <c r="X50" s="1"/>
+      <c r="Y50" s="1"/>
+      <c r="Z50" s="1"/>
+      <c r="AA50" s="1"/>
+      <c r="AB50" s="1"/>
+      <c r="AC50" s="1"/>
+      <c r="AD50" s="1"/>
+      <c r="AE50" s="1"/>
+      <c r="AF50" s="1"/>
+    </row>
+    <row r="51" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
@@ -14343,83 +14872,148 @@
       <c r="U51" s="1"/>
       <c r="V51" s="1"/>
       <c r="W51" s="1"/>
+      <c r="X51" s="1"/>
+      <c r="Y51" s="1"/>
+      <c r="Z51" s="1"/>
+      <c r="AA51" s="1"/>
+      <c r="AB51" s="1"/>
+      <c r="AC51" s="1"/>
+      <c r="AD51" s="1"/>
+      <c r="AE51" s="1"/>
+      <c r="AF51" s="1"/>
+    </row>
+    <row r="52" spans="11:32" x14ac:dyDescent="0.2">
+      <c r="K52" s="1"/>
+      <c r="L52" s="1"/>
+      <c r="M52" s="1"/>
+      <c r="N52" s="1"/>
+      <c r="O52" s="1"/>
+      <c r="P52" s="1"/>
+      <c r="Q52" s="1"/>
+      <c r="R52" s="1"/>
+      <c r="S52" s="1"/>
+      <c r="T52" s="1"/>
+      <c r="U52" s="1"/>
+      <c r="V52" s="1"/>
+      <c r="W52" s="1"/>
+      <c r="X52" s="1"/>
+      <c r="Y52" s="1"/>
+      <c r="Z52" s="1"/>
+      <c r="AA52" s="1"/>
+      <c r="AB52" s="1"/>
+      <c r="AC52" s="1"/>
+      <c r="AD52" s="1"/>
+      <c r="AE52" s="1"/>
+      <c r="AF52" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="C8:O8"/>
-    <mergeCell ref="R8:W8"/>
-    <mergeCell ref="AF8:AG8"/>
-    <mergeCell ref="X8:AE8"/>
+  <mergeCells count="3">
+    <mergeCell ref="AA9:AF9"/>
+    <mergeCell ref="AG9:AN9"/>
+    <mergeCell ref="C9:Z9"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:I51">
-    <cfRule type="expression" dxfId="14" priority="16">
-      <formula>$E10="pow"</formula>
+  <conditionalFormatting sqref="F11:K52 AB11:AF52">
+    <cfRule type="expression" dxfId="21" priority="4">
+      <formula>$E11="hb"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="20" priority="5">
+      <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G10:G51">
-    <cfRule type="expression" dxfId="13" priority="5">
-      <formula>$E10="cp"</formula>
+  <conditionalFormatting sqref="F11:L52">
+    <cfRule type="expression" dxfId="19" priority="17">
+      <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H10:I51">
-    <cfRule type="expression" dxfId="12" priority="4">
-      <formula>$E10="mc"</formula>
+  <conditionalFormatting sqref="G11:G52">
+    <cfRule type="expression" dxfId="18" priority="6">
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J10:K51">
-    <cfRule type="expression" dxfId="11" priority="6">
-      <formula>$E10="cp"</formula>
+  <conditionalFormatting sqref="H11:I52">
+    <cfRule type="expression" dxfId="17" priority="7">
+      <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L10:O51">
-    <cfRule type="expression" dxfId="10" priority="19">
-      <formula>AND($E10&lt;&gt;"",$E10&lt;&gt;"pow")</formula>
+  <conditionalFormatting sqref="J11:K52">
+    <cfRule type="expression" dxfId="16" priority="8">
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q10:Q51">
-    <cfRule type="expression" dxfId="9" priority="20">
-      <formula>AND($P10&lt;&gt;"",$P10&lt;&gt;"ru")</formula>
+  <conditionalFormatting sqref="O11:P52">
+    <cfRule type="expression" dxfId="15" priority="18">
+      <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S10:U51">
-    <cfRule type="expression" dxfId="8" priority="21">
-      <formula>$E10="pow"</formula>
+  <conditionalFormatting sqref="P11:P52">
+    <cfRule type="expression" dxfId="14" priority="11">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T10:T51">
-    <cfRule type="expression" dxfId="7" priority="8">
-      <formula>$E10="cp"</formula>
+  <conditionalFormatting sqref="S11:V52">
+    <cfRule type="expression" dxfId="13" priority="9">
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U10:U51">
-    <cfRule type="expression" dxfId="6" priority="15">
-      <formula>$E10="mc"</formula>
+  <conditionalFormatting sqref="W11:Z52">
+    <cfRule type="expression" dxfId="12" priority="10">
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V10:W51">
-    <cfRule type="expression" dxfId="5" priority="10">
-      <formula>$E10="cp"</formula>
+  <conditionalFormatting sqref="AB11:AF52">
+    <cfRule type="expression" dxfId="11" priority="19">
+      <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB10:AC101">
-    <cfRule type="expression" dxfId="4" priority="2">
-      <formula>$AA10="vg"</formula>
+  <conditionalFormatting sqref="AC11:AC52">
+    <cfRule type="expression" dxfId="10" priority="12">
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AD10:AE101">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>$AA10="lf"</formula>
+  <conditionalFormatting sqref="AD11:AD52">
+    <cfRule type="expression" dxfId="9" priority="13">
+      <formula>$E11="mc"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE11:AF52">
+    <cfRule type="expression" dxfId="8" priority="14">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK11:AL52">
+    <cfRule type="expression" dxfId="7" priority="15">
+      <formula>OR($AJ11="vg",$AJ11="gard")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM11:AN52">
+    <cfRule type="expression" dxfId="6" priority="16">
+      <formula>$AJ11="lf"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="5" priority="2">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E10:E51" xr:uid="{374AFD2C-B540-DD4B-A245-8B781F76E64C}">
-      <formula1>$C$3:$C$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11:E52" xr:uid="{374AFD2C-B540-DD4B-A245-8B781F76E64C}">
+      <formula1>$C$3:$C$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P10:P51" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
-      <formula1>$K$3:$K$6</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ11:AJ102" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
+      <formula1>$AJ$3:$AJ$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA10:AA101" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
-      <formula1>$AA$3:$AA$4</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O11:O52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
+      <formula1>$O$3:$O$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14457,268 +15051,266 @@
         <v>46</v>
       </c>
       <c r="B2" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>93</v>
+        <v>0</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="53" t="inlineStr">
-        <is>
-          <t>Profile Line #1</t>
-        </is>
-      </c>
-      <c r="B4" s="53"/>
-      <c r="D4" s="53" t="s">
+      <c r="A4" s="54" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="54"/>
+      <c r="D4" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="53"/>
-      <c r="G4" s="53" t="s">
+      <c r="E4" s="54"/>
+      <c r="G4" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="53"/>
-      <c r="J4" s="53" t="s">
+      <c r="H4" s="54"/>
+      <c r="J4" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="53"/>
-      <c r="M4" s="53" t="s">
+      <c r="K4" s="54"/>
+      <c r="M4" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="53"/>
-      <c r="P4" s="53" t="s">
+      <c r="N4" s="54"/>
+      <c r="P4" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="53"/>
+      <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="53" t="s">
+      <c r="S4" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="53"/>
+      <c r="T4" s="54"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="53" t="s">
+      <c r="V4" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="53"/>
+      <c r="W4" s="54"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="53" t="s">
+      <c r="Y4" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="53"/>
+      <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="53" t="s">
+      <c r="AB4" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="53"/>
-      <c r="AE4" s="53" t="s">
+      <c r="AC4" s="54"/>
+      <c r="AE4" s="54" t="s">
+        <v>108</v>
+      </c>
+      <c r="AF4" s="54"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="54" t="s">
+        <v>109</v>
+      </c>
+      <c r="AI4" s="54"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="54" t="s">
+        <v>110</v>
+      </c>
+      <c r="AL4" s="54"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="AF4" s="53"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="53" t="s">
+      <c r="AO4" s="54"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="54" t="s">
         <v>112</v>
       </c>
-      <c r="AI4" s="53"/>
-      <c r="AJ4" s="1"/>
-      <c r="AK4" s="53" t="s">
-        <v>113</v>
-      </c>
-      <c r="AL4" s="53"/>
-      <c r="AM4" s="1"/>
-      <c r="AN4" s="53" t="s">
-        <v>114</v>
-      </c>
-      <c r="AO4" s="53"/>
-      <c r="AP4" s="1"/>
-      <c r="AQ4" s="53" t="s">
-        <v>115</v>
-      </c>
-      <c r="AR4" s="53"/>
+      <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="42">
+      <c r="A5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="37">
         <v>1</v>
       </c>
-      <c r="D5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="E5" s="42">
+      <c r="D5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" s="37">
         <v>2</v>
       </c>
-      <c r="G5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="H5" s="42">
+      <c r="G5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" s="37">
         <v>3</v>
       </c>
-      <c r="J5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="K5" s="42">
+      <c r="J5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="K5" s="37">
         <v>4</v>
       </c>
-      <c r="M5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="N5" s="42">
+      <c r="M5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="N5" s="37">
         <v>5</v>
       </c>
-      <c r="P5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="Q5" s="42">
+      <c r="P5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q5" s="37">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
-      <c r="S5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="T5" s="42">
+      <c r="S5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="T5" s="37">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
-      <c r="V5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="W5" s="42">
+      <c r="V5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="W5" s="37">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
-      <c r="Y5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z5" s="42">
+      <c r="Y5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z5" s="37">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
-      <c r="AB5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="AC5" s="42">
+      <c r="AB5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AC5" s="37">
         <v>10</v>
       </c>
-      <c r="AE5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="AF5" s="42">
+      <c r="AE5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF5" s="37">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
-      <c r="AH5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="AI5" s="42">
+      <c r="AH5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AI5" s="37">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
-      <c r="AK5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="AL5" s="42">
+      <c r="AK5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AL5" s="37">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
-      <c r="AN5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="AO5" s="42">
+      <c r="AN5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AO5" s="37">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
-      <c r="AQ5" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="AR5" s="42">
+      <c r="AQ5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AR5" s="37">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="54" t="str">
+      <c r="A6" s="52" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="55"/>
-      <c r="D6" s="54" t="str">
+      <c r="B6" s="53"/>
+      <c r="D6" s="52" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="55"/>
-      <c r="G6" s="54" t="str">
+      <c r="E6" s="53"/>
+      <c r="G6" s="52" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="55"/>
-      <c r="J6" s="54" t="str">
+      <c r="H6" s="53"/>
+      <c r="J6" s="52" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="55"/>
-      <c r="M6" s="54" t="str">
+      <c r="K6" s="53"/>
+      <c r="M6" s="52" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="55"/>
-      <c r="P6" s="54" t="str">
+      <c r="N6" s="53"/>
+      <c r="P6" s="52" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="55"/>
+      <c r="Q6" s="53"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="54" t="str">
+      <c r="S6" s="52" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="55"/>
+      <c r="T6" s="53"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="54" t="str">
+      <c r="V6" s="52" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="55"/>
+      <c r="W6" s="53"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="54" t="str">
+      <c r="Y6" s="52" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="55"/>
+      <c r="Z6" s="53"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="54" t="str">
+      <c r="AB6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="55"/>
-      <c r="AE6" s="54" t="str">
+      <c r="AC6" s="53"/>
+      <c r="AE6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="55"/>
+      <c r="AF6" s="53"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="54" t="str">
+      <c r="AH6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="55"/>
+      <c r="AI6" s="53"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="54" t="str">
+      <c r="AK6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="55"/>
+      <c r="AL6" s="53"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="54" t="str">
+      <c r="AN6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="55"/>
+      <c r="AO6" s="53"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="54" t="str">
+      <c r="AQ6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="55"/>
+      <c r="AR6" s="53"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -14822,7 +15414,7 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="B8" s="3">
         <v>7.3</v>
@@ -15646,36 +16238,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15708,264 +16300,264 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
-        <v>169</v>
+      <c r="A2" s="24" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="54" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="54"/>
+      <c r="D4" s="54" t="s">
+        <v>138</v>
+      </c>
+      <c r="E4" s="54"/>
+      <c r="G4" s="54" t="s">
+        <v>139</v>
+      </c>
+      <c r="H4" s="54"/>
+      <c r="J4" s="54" t="s">
+        <v>140</v>
+      </c>
+      <c r="K4" s="54"/>
+      <c r="M4" s="54" t="s">
+        <v>141</v>
+      </c>
+      <c r="N4" s="54"/>
+      <c r="P4" s="54" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q4" s="54"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="54" t="s">
+        <v>143</v>
+      </c>
+      <c r="T4" s="54"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="54" t="s">
+        <v>144</v>
+      </c>
+      <c r="W4" s="54"/>
+      <c r="X4" s="1"/>
+      <c r="Y4" s="54" t="s">
+        <v>145</v>
+      </c>
+      <c r="Z4" s="54"/>
+      <c r="AA4" s="1"/>
+      <c r="AB4" s="54" t="s">
+        <v>146</v>
+      </c>
+      <c r="AC4" s="54"/>
+      <c r="AE4" s="54" t="s">
+        <v>147</v>
+      </c>
+      <c r="AF4" s="54"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="54" t="s">
+        <v>148</v>
+      </c>
+      <c r="AI4" s="54"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="54" t="s">
+        <v>149</v>
+      </c>
+      <c r="AL4" s="54"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="54" t="s">
         <v>150</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="D4" s="53" t="s">
+      <c r="AO4" s="54"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="54" t="s">
         <v>151</v>
       </c>
-      <c r="E4" s="53"/>
-      <c r="G4" s="53" t="s">
-        <v>152</v>
-      </c>
-      <c r="H4" s="53"/>
-      <c r="J4" s="53" t="s">
-        <v>153</v>
-      </c>
-      <c r="K4" s="53"/>
-      <c r="M4" s="53" t="s">
-        <v>154</v>
-      </c>
-      <c r="N4" s="53"/>
-      <c r="P4" s="53" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q4" s="53"/>
-      <c r="R4" s="1"/>
-      <c r="S4" s="53" t="s">
-        <v>156</v>
-      </c>
-      <c r="T4" s="53"/>
-      <c r="U4" s="1"/>
-      <c r="V4" s="53" t="s">
-        <v>157</v>
-      </c>
-      <c r="W4" s="53"/>
-      <c r="X4" s="1"/>
-      <c r="Y4" s="53" t="s">
-        <v>158</v>
-      </c>
-      <c r="Z4" s="53"/>
-      <c r="AA4" s="1"/>
-      <c r="AB4" s="53" t="s">
-        <v>159</v>
-      </c>
-      <c r="AC4" s="53"/>
-      <c r="AE4" s="53" t="s">
-        <v>160</v>
-      </c>
-      <c r="AF4" s="53"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="53" t="s">
-        <v>161</v>
-      </c>
-      <c r="AI4" s="53"/>
-      <c r="AJ4" s="1"/>
-      <c r="AK4" s="53" t="s">
-        <v>162</v>
-      </c>
-      <c r="AL4" s="53"/>
-      <c r="AM4" s="1"/>
-      <c r="AN4" s="53" t="s">
-        <v>163</v>
-      </c>
-      <c r="AO4" s="53"/>
-      <c r="AP4" s="1"/>
-      <c r="AQ4" s="53" t="s">
-        <v>164</v>
-      </c>
-      <c r="AR4" s="53"/>
+      <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="44">
+      <c r="A5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="39">
         <v>1</v>
       </c>
-      <c r="D5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="E5" s="44">
+      <c r="D5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" s="39">
         <v>2</v>
       </c>
-      <c r="G5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="H5" s="44">
+      <c r="G5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" s="39">
         <v>3</v>
       </c>
-      <c r="J5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="K5" s="44">
+      <c r="J5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="K5" s="39">
         <v>4</v>
       </c>
-      <c r="M5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="N5" s="44">
+      <c r="M5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="N5" s="39">
         <v>5</v>
       </c>
-      <c r="P5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="Q5" s="44">
+      <c r="P5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q5" s="39">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
-      <c r="S5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="T5" s="44">
+      <c r="S5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="T5" s="39">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
-      <c r="V5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="W5" s="44">
+      <c r="V5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="W5" s="39">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
-      <c r="Y5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z5" s="44">
+      <c r="Y5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z5" s="39">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
-      <c r="AB5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="AC5" s="44">
+      <c r="AB5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AC5" s="39">
         <v>10</v>
       </c>
-      <c r="AE5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="AF5" s="44">
+      <c r="AE5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF5" s="39">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
-      <c r="AH5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="AI5" s="44">
+      <c r="AH5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AI5" s="39">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
-      <c r="AK5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="AL5" s="44">
+      <c r="AK5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AL5" s="39">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
-      <c r="AN5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="AO5" s="44">
+      <c r="AN5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AO5" s="39">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
-      <c r="AQ5" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="AR5" s="44">
+      <c r="AQ5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AR5" s="39">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="56" t="str">
+      <c r="A6" s="55" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="57"/>
-      <c r="D6" s="56" t="str">
+      <c r="B6" s="56"/>
+      <c r="D6" s="55" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="57"/>
-      <c r="G6" s="56" t="str">
+      <c r="E6" s="56"/>
+      <c r="G6" s="55" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="57"/>
-      <c r="J6" s="56" t="str">
+      <c r="H6" s="56"/>
+      <c r="J6" s="55" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="57"/>
-      <c r="M6" s="56" t="str">
+      <c r="K6" s="56"/>
+      <c r="M6" s="55" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="57"/>
-      <c r="P6" s="56" t="str">
+      <c r="N6" s="56"/>
+      <c r="P6" s="55" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="57"/>
+      <c r="Q6" s="56"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="56" t="str">
+      <c r="S6" s="55" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="57"/>
+      <c r="T6" s="56"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="56" t="str">
+      <c r="V6" s="55" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="57"/>
+      <c r="W6" s="56"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="56" t="str">
+      <c r="Y6" s="55" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="57"/>
+      <c r="Z6" s="56"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="56" t="str">
+      <c r="AB6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="57"/>
-      <c r="AE6" s="56" t="str">
+      <c r="AC6" s="56"/>
+      <c r="AE6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="57"/>
+      <c r="AF6" s="56"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="56" t="str">
+      <c r="AH6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="57"/>
+      <c r="AI6" s="56"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="56" t="str">
+      <c r="AK6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="57"/>
+      <c r="AL6" s="56"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="56" t="str">
+      <c r="AN6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="57"/>
+      <c r="AO6" s="56"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="56" t="str">
+      <c r="AQ6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="57"/>
+      <c r="AR6" s="56"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -16869,14 +17461,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -16893,12 +17483,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16906,113 +17498,134 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E1F343-68A5-3340-AF23-43D8E7E1F914}">
-  <dimension ref="A2:G23"/>
+  <dimension ref="A2:H24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="7" customWidth="1"/>
     <col min="6" max="6" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="58" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="58"/>
-      <c r="D2" s="59" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="57" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="57"/>
+      <c r="D2" s="58" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" s="58"/>
+      <c r="G2" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="59"/>
-      <c r="G2" s="24" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="32" t="s">
+        <v>196</v>
+      </c>
+      <c r="B3" s="33"/>
+      <c r="D3" s="34" t="s">
+        <v>196</v>
+      </c>
+      <c r="E3" s="35"/>
+      <c r="G3" s="22"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G4" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G6" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="H6" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="D16" s="4"/>
@@ -17060,11 +17673,22 @@
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
     </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="D2:E2"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3 E3" xr:uid="{62365587-5741-D749-B74F-CDA32F05212C}">
+      <formula1>$G$5:$G$6</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -17084,10 +17708,10 @@
         <v>25</v>
       </c>
       <c r="B2" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="13" t="s">
         <v>61</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>62</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>29</v>
@@ -17102,7 +17726,7 @@
         <v>28</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>30</v>
@@ -17116,10 +17740,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>130.0</v>
+        <v>130</v>
       </c>
       <c r="C3" s="3">
-        <v>60.0</v>
+        <v>60</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
@@ -17169,10 +17793,10 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="J5" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -17344,10 +17968,10 @@
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
+        <v>75</v>
+      </c>
+      <c r="F5" t="s">
         <v>76</v>
-      </c>
-      <c r="F5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -17470,36 +18094,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="60" t="s">
+      <c r="B2" s="59" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="F2" s="59" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="J2" s="59" t="s">
+        <v>123</v>
+      </c>
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="N2" s="59" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="F2" s="60" t="s">
+      <c r="O2" s="59"/>
+      <c r="P2" s="59"/>
+      <c r="R2" s="59" t="s">
         <v>125</v>
       </c>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="J2" s="60" t="s">
+      <c r="S2" s="59"/>
+      <c r="T2" s="59"/>
+      <c r="V2" s="59" t="s">
         <v>126</v>
       </c>
-      <c r="K2" s="60"/>
-      <c r="L2" s="60"/>
-      <c r="N2" s="60" t="s">
-        <v>127</v>
-      </c>
-      <c r="O2" s="60"/>
-      <c r="P2" s="60"/>
-      <c r="R2" s="60" t="s">
-        <v>128</v>
-      </c>
-      <c r="S2" s="60"/>
-      <c r="T2" s="60"/>
-      <c r="V2" s="60" t="s">
-        <v>129</v>
-      </c>
-      <c r="W2" s="60"/>
-      <c r="X2" s="60"/>
+      <c r="W2" s="59"/>
+      <c r="X2" s="59"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>